<commit_message>
eval(s83): corrección FAAST FLEX (Xtralis) ≠ FAAST LT-200 (System Sensor)
Alberto cazó que la 2ª pasada fusionó dos familias DISTINTAS (distinto OEM)
porque ambas se llaman "FAAST". El lumping estaba en 2 agentes (Notifier metió
NFXI-FLX en LT-200; Morley metió MI-FLX-010). Mi "FAAST reconciliado" fue
over-claim.

Overlay de correcciones humanas (evals/s83_family_corrections.json, durable,
crece con la review): FLEX (NFXI-FLX/MI-FLX-010/FLX-010/FAAST FLEX) → familia
Xtralis; resto → FAAST LT-200 (System Sensor); 8100-series flagged para revisión.
Excel regenerado.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s83_familias_para_revisar.xlsx
+++ b/s83_familias_para_revisar.xlsx
@@ -447,7 +447,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -6542,7 +6542,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -8132,7 +8132,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -9014,7 +9014,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>FAAST aspirating smoke detection (ASD) series</t>
+          <t>FAAST FLEX (aspiracion SMB, Xtralis)</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -9032,7 +9032,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>FAAST = aspirating smoke detection (System Sensor/Xtralis OEM) sold under Morley/Notifier (project ground-truth reference_faast). FAAST LT (LT-200 series) and bare FAAST are the Morley-branded aspirating units; MI-FLX-010 = Morley-coded FAAST FLEX (FLX-010) variant. Distinct standalone-vs-addressabl</t>
+          <t>Alberto s83: FAAST FLEX = Xtralis, familia DISTINTA de FAAST LT-200 (System Sensor) aunque ambas se llamen FAAST</t>
         </is>
       </c>
     </row>
@@ -11162,7 +11162,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -11492,7 +11492,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -11522,7 +11522,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -12092,7 +12092,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -12122,7 +12122,7 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -12134,17 +12134,17 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>FAAST LT-200 / ASD (aspiración, OEM System Sensor vendida por Notifier)</t>
+          <t>FAAST 8100 (aspiracion) - REVISAR: System Sensor XM-8100 vs Xtralis FLEX?</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>NFXI-BSF-WCH</t>
-        </is>
-      </c>
-      <c r="D390" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>FAAST-8100E</t>
+        </is>
+      </c>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
       <c r="E390" t="n">
@@ -12152,7 +12152,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Ground-truth: NFXI-ASD11/12/22 = aspiración FAAST LT-200 (OEM System Sensor, vendida por Notifier). FAAST LT-200/LT-200/FAAST-LT = serie LT-200; LTS-240 = variante de la serie; FAAST-8100E = FAAST 8100 (aspiración de mayor canal); NFXI-FLX = FAAST FLEX (Xtralis OEM bajo Notifier); ASD11 = NFXI-ASD11</t>
+          <t>Alberto s83: separar de LT-200; serie 8100 ambigua -&gt; confirmar</t>
         </is>
       </c>
     </row>
@@ -12164,7 +12164,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>FAAST LT-200 / ASD (aspiración, OEM System Sensor vendida por Notifier)</t>
+          <t>FAAST FLEX (aspiracion SMB, Xtralis)</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Ground-truth: NFXI-ASD11/12/22 = aspiración FAAST LT-200 (OEM System Sensor, vendida por Notifier). FAAST LT-200/LT-200/FAAST-LT = serie LT-200; LTS-240 = variante de la serie; FAAST-8100E = FAAST 8100 (aspiración de mayor canal); NFXI-FLX = FAAST FLEX (Xtralis OEM bajo Notifier); ASD11 = NFXI-ASD11</t>
+          <t>Alberto s83: FAAST FLEX = Xtralis, familia DISTINTA de FAAST LT-200 (System Sensor) aunque ambas se llamen FAAST</t>
         </is>
       </c>
     </row>
@@ -12199,7 +12199,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>ASD11</t>
+          <t>NFXI-BSF-WCH</t>
         </is>
       </c>
       <c r="D392" s="2" t="inlineStr">
@@ -12229,7 +12229,7 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>FAAST-8100E</t>
+          <t>ASD11</t>
         </is>
       </c>
       <c r="D393" s="2" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -13412,7 +13412,7 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -14342,7 +14342,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -15362,7 +15362,7 @@
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -17462,7 +17462,7 @@
       </c>
       <c r="F567" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -17492,7 +17492,7 @@
       </c>
       <c r="F568" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -18122,7 +18122,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -18212,7 +18212,7 @@
       </c>
       <c r="F592" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -18974,7 +18974,7 @@
       </c>
       <c r="B618" t="inlineStr">
         <is>
-          <t>FAAST aspirating smoke detection (XM-8100 series)</t>
+          <t>FAAST 8100 (aspiracion) - REVISAR: System Sensor XM-8100 vs Xtralis FLEX?</t>
         </is>
       </c>
       <c r="C618" t="inlineStr">
@@ -18982,9 +18982,9 @@
           <t>XM-8100E</t>
         </is>
       </c>
-      <c r="D618" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
+      <c r="D618" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
       <c r="E618" t="n">
@@ -18992,7 +18992,7 @@
       </c>
       <c r="F618" t="inlineStr">
         <is>
-          <t>XM-8100E = FAAST XM 8100, conventional aspirating smoke detector (ASD), dual-source blue-LED + IR laser. System Sensor is the OEM of FAAST (project ground-truth). Distinct FAAST series from the LT-200 (this is the larger 8100 series). Source: environmental-expert.com FAAST XM 8100 listing + Honeywel</t>
+          <t>Alberto s83: separar de LT-200; serie 8100 ambigua -&gt; confirmar</t>
         </is>
       </c>
     </row>
@@ -19412,7 +19412,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19442,7 +19442,7 @@
       </c>
       <c r="F633" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19484,7 +19484,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>FAAST FLEX (aspiracion SMB)</t>
+          <t>FAAST FLEX (aspiracion SMB, Xtralis)</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>Web (xtralis.com, honeywell.com): FLX-010 = unidad FAAST FLEX de un canal (FLX-020 = doble canal). Mismo producto base. Ground-truth proyecto: FAAST FLEX = deteccion por aspiracion Xtralis (familia aparte de VESDA).</t>
+          <t>Alberto s83: FAAST FLEX = Xtralis, familia DISTINTA de FAAST LT-200 (System Sensor) aunque ambas se llamen FAAST</t>
         </is>
       </c>
     </row>
@@ -19514,7 +19514,7 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>FAAST FLEX (aspiracion SMB)</t>
+          <t>FAAST FLEX (aspiracion SMB, Xtralis)</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="F636" t="inlineStr">
         <is>
-          <t>Web (xtralis.com, honeywell.com): FLX-010 = unidad FAAST FLEX de un canal (FLX-020 = doble canal). Mismo producto base. Ground-truth proyecto: FAAST FLEX = deteccion por aspiracion Xtralis (familia aparte de VESDA).</t>
+          <t>Alberto s83: FAAST FLEX = Xtralis, familia DISTINTA de FAAST LT-200 (System Sensor) aunque ambas se llamen FAAST</t>
         </is>
       </c>
     </row>
@@ -19742,7 +19742,7 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19772,7 +19772,7 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19802,7 +19802,7 @@
       </c>
       <c r="F645" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19832,7 +19832,7 @@
       </c>
       <c r="F646" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19862,7 +19862,7 @@
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19892,7 +19892,7 @@
       </c>
       <c r="F648" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19922,7 +19922,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>
@@ -19952,7 +19952,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>no agrupado en la 2a pasada (singleton/no-match)</t>
+          <t>no agrupado en la 2a pasada</t>
         </is>
       </c>
     </row>

</xml_diff>